<commit_message>
Fix title screen VO
</commit_message>
<xml_diff>
--- a/VO_Manifest.xlsx
+++ b/VO_Manifest.xlsx
@@ -448,12 +448,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>vo_review_landing</t>
+          <t>vo_review_landing_v2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>नमस्ते दोस्त, मैं हूँ स्विफ़्टी। आज हम एक कहानी पढ़ेंगे—कालू-मालू-आलू।</t>
+          <t>नमस्ते दोस्त, मैं हूँ स्विफ़्टी। आज हम एक कहानी पढ़ेंगे—आलू-मालू-कालू।</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1276,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>sfx_puppy_bark</t>
+          <t>sfx_dog_bark</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SFX (असली रिकॉर्डिंग, AI नहीं): छोटे पिल्ले की 3 प्यारी, पतली भौंक — भौं, भौं, भौं (~0.8 सेकंड)। कहानी पेज 8 पर VO “…उसे सुनाई दिया,” के तुरंत बाद बजती है। स्रोत: freesound.org/s/591137 (dtmendes, cockapoo puppy), लाइसेंस CC0; पिच थोड़ी ऊँची की गई।</t>
+          <t>SFX (असली रिकॉर्डिंग, AI नहीं): बड़े कुत्ते (St. Bernard) की 3 भारी भौंक — भौं, भौं, भौं (~1.3 सेकंड)। कहानी पेज 8 पर VO “…उसे सुनाई दिया,” के तुरंत बाद बजती है। स्रोत: freesound.org/s/784914 (Primitv094), लाइसेंस CC0।</t>
         </is>
       </c>
     </row>

</xml_diff>